<commit_message>
Rename Excel case Meta sheet to Settings and refresh docs.
Use Settings tab and read_settings/read_settings_role in excel_ds_test_runner; update TC08 workbook, unit tests, and architecture doc.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/DataValidation/GC/TC08_CRDC-VerifyInvalidIntegerValue.xlsx
+++ b/tests/DataValidation/GC/TC08_CRDC-VerifyInvalidIntegerValue.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Steps" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,8 +461,6 @@
           <t>open_data_submissions</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -475,7 +473,6 @@
           <t>New|metadata only|GC|autoQA - AutomationQA_Study</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -488,7 +485,6 @@
           <t>TC08</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -496,8 +492,6 @@
           <t>click_validate</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">

</xml_diff>